<commit_message>
Score per control, not per region (v2.1.0)
A real 17-region scan reported 144 failures because each regional check
counted once per region: one control off in 16 unused regions showed as
16 failures. Results now roll up to one verdict per control (fails if it
fails in any region, names the regions); score and counts use controls.
Per-region results and evidence are unchanged.

- summary: new `checks` (per control) and `result_counts` (per region)
- HTML report and workbook lead with controls; workbook adds Region Detail
- Demo page rolls up client-side, so v2.0.0 report.json files still open
- Tests for roll-up precedence and multi-region verdicts

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017pwRQCbGzSVKnLyfg31ziv
</commit_message>
<xml_diff>
--- a/web/sample/workbook.xlsx
+++ b/web/sample/workbook.xlsx
@@ -8,17 +8,19 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Automated Checks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Failed Resources" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual Controls" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criteria Coverage" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Region Detail" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Failed Resources" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual Controls" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criteria Coverage" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Automated Checks'!$A$1:$J$48</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Failed Resources'!$A$1:$F$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Manual Controls'!$A$1:$I$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Criteria Coverage'!$A$1:$H$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Controls'!$A$1:$H$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Region Detail'!$A$1:$G$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Failed Resources'!$A$1:$F$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Manual Controls'!$A$1:$I$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Criteria Coverage'!$A$1:$H$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -470,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -533,7 +535,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:42:50Z</t>
+          <t>2026-10-26T15:22:10Z</t>
         </is>
       </c>
     </row>
@@ -545,7 +547,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:42:53Z</t>
+          <t>2026-10-26T15:22:13Z</t>
         </is>
       </c>
     </row>
@@ -557,48 +559,60 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>42% of evaluated checks passing</t>
+          <t>27% of evaluated controls passing</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Pass / Fail / Error / N/A</t>
+          <t>Controls: pass / fail / error / N/A</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>16 / 22 / 2 / 7</t>
+          <t>8 / 22 / 1 / 0</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Tool</t>
+          <t>Region-level results</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>soc2kit 2.0.0</t>
+          <t>47</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Tool</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>soc2kit 2.1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Automated technical evidence only. Criteria mappings are guidance; your auditor determines control sufficiency. Most SOC 2 controls are procedural - see manual_controls.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B10"/>
+  <autoFilter ref="A1:B11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -609,19 +623,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -647,32 +659,22 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Region</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Result</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>Remediation</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Remediation</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Evidence file</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Evaluated (UTC)</t>
+          <t>Evidence files</t>
         </is>
       </c>
     </row>
@@ -697,34 +699,24 @@
           <t>CRITICAL</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>us-east-1</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>1 of 2 resources fail (us-east-1)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>1 of 2 failing</t>
+          <t>Set PubliclyAccessible to false and place the instance in private subnets.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Set PubliclyAccessible to false and place the instance in private subnets.</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>evidence/DATA-07__us-east-1.json</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
+          <t>evidence/DATA-07__us-east-1.json, evidence/DATA-07__us-west-2.json</t>
         </is>
       </c>
     </row>
@@ -749,34 +741,24 @@
           <t>CRITICAL</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>global</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 failing</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>1 of 1 failing</t>
+          <t>Sign in as root and enable a hardware or virtual MFA device under Security credentials.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Sign in as root and enable a hardware or virtual MFA device under Security credentials.</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
           <t>evidence/IAM-01.json</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
         </is>
       </c>
     </row>
@@ -801,34 +783,24 @@
           <t>CRITICAL</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>us-east-1</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>1 of 4 resources fail (us-east-1)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>1 of 3 failing</t>
+          <t>Remove the open rule; use SSM Session Manager or a VPN / bastion with a narrow source range.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Remove the open rule; use SSM Session Manager or a VPN / bastion with a narrow source range.</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>evidence/NET-01__us-east-1.json</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
+          <t>evidence/NET-01__us-east-1.json, evidence/NET-01__us-west-2.json</t>
         </is>
       </c>
     </row>
@@ -853,34 +825,24 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>us-east-1</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>1 of 2 resources fail (us-east-1)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>1 of 2 failing</t>
+          <t>Set BackupRetentionPeriod to 7 or more.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Set BackupRetentionPeriod to 7 or more.</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>evidence/AVL-01__us-east-1.json</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
+          <t>evidence/AVL-01__us-east-1.json, evidence/AVL-01__us-west-2.json</t>
         </is>
       </c>
     </row>
@@ -905,34 +867,24 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>us-east-1</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>1 of 2 resources fail (us-east-1)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>1 of 2 failing</t>
+          <t>Encryption can't be turned on in place: snapshot, copy the snapshot with encryption, restore.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Encryption can't be turned on in place: snapshot, copy the snapshot with encryption, restore.</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>evidence/DATA-06__us-east-1.json</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
+          <t>evidence/DATA-06__us-east-1.json, evidence/DATA-06__us-west-2.json</t>
         </is>
       </c>
     </row>
@@ -957,34 +909,24 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>global</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>1 of 2 failing</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>1 of 2 failing</t>
+          <t>Enable MFA for each listed user, or remove their console password and use IAM Identity Center.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Enable MFA for each listed user, or remove their console password and use IAM Identity Center.</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
           <t>evidence/IAM-04.json</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:53Z</t>
         </is>
       </c>
     </row>
@@ -1009,34 +951,24 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>global</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>1 of 2 failing</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>1 of 2 failing</t>
+          <t>Replace '*:*' with the specific actions and resources the principal needs.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Replace '*:*' with the specific actions and resources the principal needs.</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
           <t>evidence/IAM-08.json</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
         </is>
       </c>
     </row>
@@ -1061,34 +993,24 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>us-west-2</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Fails in 1 of 2 regions (us-west-2)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>1 of 1 failing</t>
+          <t>Enable AWS Config in this region, recording all resource types.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Enable AWS Config in this region, recording all resource types.</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>evidence/LOG-04__us-west-2.json</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
+          <t>evidence/LOG-04__us-east-1.json, evidence/LOG-04__us-west-2.json</t>
         </is>
       </c>
     </row>
@@ -1113,34 +1035,24 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>us-west-2</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Fails in 1 of 2 regions (us-west-2)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>1 of 1 failing</t>
+          <t>Enable GuardDuty in this region (ideally org-wide with a delegated admin).</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Enable GuardDuty in this region (ideally org-wide with a delegated admin).</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>evidence/LOG-05__us-west-2.json</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
+          <t>evidence/LOG-05__us-east-1.json, evidence/LOG-05__us-west-2.json</t>
         </is>
       </c>
     </row>
@@ -1165,34 +1077,24 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>us-east-1</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>1 of 2 resources fail (us-east-1)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>1 of 2 failing</t>
+          <t>Modify the instance to enable Multi-AZ (dev/test databases can be accepted as a documented exception).</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Modify the instance to enable Multi-AZ (dev/test databases can be accepted as a documented exception).</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>evidence/AVL-02__us-east-1.json</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:52Z</t>
+          <t>evidence/AVL-02__us-east-1.json, evidence/AVL-02__us-west-2.json</t>
         </is>
       </c>
     </row>
@@ -1217,34 +1119,24 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>us-west-2</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Fails in 1 of 2 regions (us-west-2)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>1 of 1 failing</t>
+          <t>Create an AWS Backup plan covering production resources in this region.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Create an AWS Backup plan covering production resources in this region.</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>evidence/AVL-03__us-west-2.json</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:50Z</t>
+          <t>evidence/AVL-03__us-east-1.json, evidence/AVL-03__us-west-2.json</t>
         </is>
       </c>
     </row>
@@ -1269,34 +1161,24 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>global</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>1 of 4 failing</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>1 of 4 failing</t>
+          <t>Add a Deny statement for "s3:*" with Condition {"Bool": {"aws:SecureTransport": "false"}}.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Add a Deny statement for "s3:*" with Condition {"Bool": {"aws:SecureTransport": "false"}}.</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
           <t>evidence/DATA-03.json</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
         </is>
       </c>
     </row>
@@ -1321,34 +1203,24 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>us-west-2</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Fails in 1 of 2 regions (us-west-2)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>1 of 1 failing</t>
+          <t>Enable EBS encryption by default in this region.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Enable EBS encryption by default in this region.</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>evidence/DATA-05__us-west-2.json</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:50Z</t>
+          <t>evidence/DATA-05__us-east-1.json, evidence/DATA-05__us-west-2.json</t>
         </is>
       </c>
     </row>
@@ -1373,34 +1245,24 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>us-east-1</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>1 of 2 resources fail (us-east-1)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>1 of 2 failing</t>
+          <t>Enable automatic key rotation on the key.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Enable automatic key rotation on the key.</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>evidence/DATA-08__us-east-1.json</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
+          <t>evidence/DATA-08__us-east-1.json, evidence/DATA-08__us-west-2.json</t>
         </is>
       </c>
     </row>
@@ -1425,34 +1287,24 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>global</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 failing</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>1 of 1 failing</t>
+          <t>Set an account password policy: minimum length 14, require upper/lower/number/symbol, prevent reuse of 24.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Set an account password policy: minimum length 14, require upper/lower/number/symbol, prevent reuse of 24.</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
           <t>evidence/IAM-03.json</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
         </is>
       </c>
     </row>
@@ -1477,34 +1329,24 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>us-west-2</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>1 of 2 resources fail (us-west-2)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>1 of 1 failing</t>
+          <t>Enable Security Hub with the AWS Foundational Security Best Practices standard.</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Enable Security Hub with the AWS Foundational Security Best Practices standard.</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>evidence/LOG-06__us-west-2.json</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:52Z</t>
+          <t>evidence/LOG-06__us-east-1.json, evidence/LOG-06__us-west-2.json</t>
         </is>
       </c>
     </row>
@@ -1529,34 +1371,24 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>us-west-2</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>1 of 2 resources fail (us-west-2)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>1 of 1 failing</t>
+          <t>Enable VPC flow logs (at least REJECT traffic) to CloudWatch Logs or S3.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Enable VPC flow logs (at least REJECT traffic) to CloudWatch Logs or S3.</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>evidence/LOG-07__us-west-2.json</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
+          <t>evidence/LOG-07__us-east-1.json, evidence/LOG-07__us-west-2.json</t>
         </is>
       </c>
     </row>
@@ -1581,34 +1413,24 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>global</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>1 of 4 failing</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>1 of 4 failing</t>
+          <t>Enable versioning (and a lifecycle rule to expire old versions to control cost).</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Enable versioning (and a lifecycle rule to expire old versions to control cost).</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
           <t>evidence/DATA-04.json</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:50Z</t>
         </is>
       </c>
     </row>
@@ -1633,34 +1455,24 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>us-east-1</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 resources fail (us-east-1)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>1 of 1 failing</t>
+          <t>Configure a rotation Lambda and schedule for the secret.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Configure a rotation Lambda and schedule for the secret.</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>evidence/DATA-09__us-east-1.json</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
+          <t>evidence/DATA-09__us-east-1.json, evidence/DATA-09__us-west-2.json</t>
         </is>
       </c>
     </row>
@@ -1685,34 +1497,24 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>global</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>1 of 3 failing</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>1 of 3 failing</t>
+          <t>Move the user's policies onto a group or role and detach them from the user.</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Move the user's policies onto a group or role and detach them from the user.</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
           <t>evidence/IAM-07.json</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
         </is>
       </c>
     </row>
@@ -1737,34 +1539,24 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>global</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 failing</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>1 of 1 failing</t>
+          <t>Configure SSE-KMS on the trail with a dedicated customer-managed key.</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Configure SSE-KMS on the trail with a dedicated customer-managed key.</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
           <t>evidence/LOG-03.json</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
         </is>
       </c>
     </row>
@@ -1789,34 +1581,24 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>us-east-1</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>1 of 2 resources fail (us-east-1)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>1 of 2 failing</t>
+          <t>Set retention to 365+ days (or 'never expire') on each log group.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Set retention to 365+ days (or 'never expire') on each log group.</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>evidence/LOG-08__us-east-1.json</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
+          <t>evidence/LOG-08__us-east-1.json, evidence/LOG-08__us-west-2.json</t>
         </is>
       </c>
     </row>
@@ -1841,103 +1623,83 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>us-east-1</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>ERROR</t>
         </is>
       </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Could not be evaluated in 2 region(s)</t>
+        </is>
+      </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Check could not be evaluated (The AWS simulator used for this sample does not support this API.)</t>
+          <t>Create an account- or organization-level analyzer in this region.</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Create an account- or organization-level analyzer in this region.</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>evidence/IAM-09__us-east-1.json</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
+          <t>evidence/IAM-09__us-east-1.json, evidence/IAM-09__us-west-2.json</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>IAM-09</t>
+          <t>DATA-02</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>IAM Access Analyzer is enabled</t>
+          <t>No S3 bucket allows public access</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>CC6.1, CC7.1</t>
+          <t>CC6.1, C1.1</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>us-west-2</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>ERROR</t>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>4 of 4 passing</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Check could not be evaluated (The AWS simulator used for this sample does not support this API.)</t>
+          <t>Enable Block Public Access on the bucket; serve public content through CloudFront with OAC instead.</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Create an account- or organization-level analyzer in this region.</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>evidence/IAM-09__us-west-2.json</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
+          <t>evidence/DATA-02.json</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>DATA-02</t>
+          <t>IAM-02</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>No S3 bucket allows public access</t>
+          <t>Root account has no access keys</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>CC6.1, C1.1</t>
+          <t>CC6.1</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1945,51 +1707,41 @@
           <t>CRITICAL</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>global</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>4 of 4 passing</t>
+          <t>Delete any root access keys and use IAM roles for programmatic access.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Enable Block Public Access on the bucket; serve public content through CloudFront with OAC instead.</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>evidence/DATA-02.json</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
+          <t>evidence/IAM-02.json</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>IAM-02</t>
+          <t>LOG-01</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Root account has no access keys</t>
+          <t>A multi-region CloudTrail trail is logging</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>CC6.1</t>
+          <t>CC7.2, CC7.3</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1997,1136 +1749,2044 @@
           <t>CRITICAL</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>global</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>1 of 1 passing</t>
+          <t>Create a multi-region trail (or an organization trail) delivering to a dedicated S3 bucket.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Delete any root access keys and use IAM roles for programmatic access.</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>evidence/IAM-02.json</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
+          <t>evidence/LOG-01.json</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>LOG-01</t>
+          <t>DATA-01</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>A multi-region CloudTrail trail is logging</t>
+          <t>S3 Block Public Access is on at the account level</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>CC7.2, CC7.3</t>
+          <t>CC6.1, C1.1</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>global</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>1 of 1 passing</t>
+          <t>Turn on all four Block Public Access settings for the account.</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Create a multi-region trail (or an organization trail) delivering to a dedicated S3 bucket.</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>evidence/LOG-01.json</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
+          <t>evidence/DATA-01.json</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>NET-01</t>
+          <t>IAM-05</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>No security group exposes SSH or RDP to the internet</t>
+          <t>Access keys are rotated within 90 days</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>CC6.6</t>
+          <t>CC6.1, CC6.2</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>us-west-2</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>1 of 1 passing</t>
+          <t>Rotate old keys, or better, replace long-lived keys with IAM roles / IAM Identity Center.</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Remove the open rule; use SSM Session Manager or a VPN / bastion with a narrow source range.</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>evidence/NET-01__us-west-2.json</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
+          <t>evidence/IAM-05.json</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>DATA-01</t>
+          <t>IAM-06</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>S3 Block Public Access is on at the account level</t>
+          <t>Unused credentials are disabled</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>CC6.1, C1.1</t>
+          <t>CC6.2, CC6.3</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>global</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>3 of 3 passing</t>
+        </is>
+      </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>1 of 1 passing</t>
+          <t>Disable or delete the stale password / access key; review whether the user still needs access.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Turn on all four Block Public Access settings for the account.</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>evidence/DATA-01.json</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:50Z</t>
+          <t>evidence/IAM-06.json</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>LOG-04</t>
+          <t>LOG-02</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>AWS Config is recording</t>
+          <t>CloudTrail log file validation is enabled</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>CC7.1, CC8.1</t>
+          <t>CC7.2</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>us-east-1</t>
-        </is>
-      </c>
-      <c r="F31" s="5" t="inlineStr">
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>1 of 1 passing</t>
+          <t>Enable log file validation on the trail.</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Enable AWS Config in this region, recording all resource types.</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>evidence/LOG-04__us-east-1.json</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
+          <t>evidence/LOG-02.json</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>LOG-05</t>
+          <t>NET-02</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>GuardDuty is enabled</t>
+          <t>Default security groups allow no traffic</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>CC6.8, CC7.2</t>
+          <t>CC6.6</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>us-east-1</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>All 2 resources pass</t>
+        </is>
+      </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>1 of 1 passing</t>
+          <t>Remove all inbound and outbound rules from each VPC's default security group.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Enable GuardDuty in this region (ideally org-wide with a delegated admin).</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>evidence/LOG-05__us-east-1.json</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>AVL-03</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>An AWS Backup plan exists</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>A1.2</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>us-east-1</t>
-        </is>
-      </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>1 of 1 passing</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>Create an AWS Backup plan covering production resources in this region.</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>evidence/AVL-03__us-east-1.json</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>DATA-05</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>EBS encryption by default is on</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>CC6.1, C1.1</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>us-east-1</t>
-        </is>
-      </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>1 of 1 passing</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>Enable EBS encryption by default in this region.</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>evidence/DATA-05__us-east-1.json</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:50Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>IAM-05</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Access keys are rotated within 90 days</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>CC6.1, CC6.2</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>global</t>
-        </is>
-      </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>1 of 1 passing</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>Rotate old keys, or better, replace long-lived keys with IAM roles / IAM Identity Center.</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>evidence/IAM-05.json</t>
-        </is>
-      </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>IAM-06</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Unused credentials are disabled</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>CC6.2, CC6.3</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>global</t>
-        </is>
-      </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>3 of 3 passing</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>Disable or delete the stale password / access key; review whether the user still needs access.</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>evidence/IAM-06.json</t>
-        </is>
-      </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>LOG-02</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>CloudTrail log file validation is enabled</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>CC7.2</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>global</t>
-        </is>
-      </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>1 of 1 passing</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>Enable log file validation on the trail.</t>
-        </is>
-      </c>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>evidence/LOG-02.json</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>LOG-06</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Security Hub is enabled</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>CC7.1</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>us-east-1</t>
-        </is>
-      </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>1 of 1 passing</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>Enable Security Hub with the AWS Foundational Security Best Practices standard.</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>evidence/LOG-06__us-east-1.json</t>
-        </is>
-      </c>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>LOG-07</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>Every VPC has flow logs</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>CC7.2</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>us-east-1</t>
-        </is>
-      </c>
-      <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>1 of 1 passing</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>Enable VPC flow logs (at least REJECT traffic) to CloudWatch Logs or S3.</t>
-        </is>
-      </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>evidence/LOG-07__us-east-1.json</t>
-        </is>
-      </c>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>NET-02</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>Default security groups allow no traffic</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>CC6.6</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>us-east-1</t>
-        </is>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>1 of 1 passing</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>Remove all inbound and outbound rules from each VPC's default security group.</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>evidence/NET-02__us-east-1.json</t>
-        </is>
-      </c>
-      <c r="J40" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>NET-02</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>Default security groups allow no traffic</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>CC6.6</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>us-west-2</t>
-        </is>
-      </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>1 of 1 passing</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>Remove all inbound and outbound rules from each VPC's default security group.</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>evidence/NET-02__us-west-2.json</t>
-        </is>
-      </c>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>DATA-07</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>RDS databases are not publicly accessible</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>CC6.6</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>us-west-2</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>No resources in scope</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>Set PubliclyAccessible to false and place the instance in private subnets.</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>evidence/DATA-07__us-west-2.json</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:52Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>AVL-01</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>RDS automated backups are kept at least 7 days</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>A1.2</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>us-west-2</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>No resources in scope</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>Set BackupRetentionPeriod to 7 or more.</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t>evidence/AVL-01__us-west-2.json</t>
-        </is>
-      </c>
-      <c r="J43" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>DATA-06</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>RDS databases are encrypted at rest</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>CC6.1, C1.1</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>us-west-2</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>No resources in scope</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>Encryption can't be turned on in place: snapshot, copy the snapshot with encryption, restore.</t>
-        </is>
-      </c>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t>evidence/DATA-06__us-west-2.json</t>
-        </is>
-      </c>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:52Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>AVL-02</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>RDS databases are Multi-AZ</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>A1.2</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>us-west-2</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>No resources in scope</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>Modify the instance to enable Multi-AZ (dev/test databases can be accepted as a documented exception).</t>
-        </is>
-      </c>
-      <c r="I45" s="2" t="inlineStr">
-        <is>
-          <t>evidence/AVL-02__us-west-2.json</t>
-        </is>
-      </c>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:52Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>DATA-08</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Customer-managed KMS keys rotate automatically</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>CC6.1</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>us-west-2</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>No resources in scope</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>Enable automatic key rotation on the key.</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>evidence/DATA-08__us-west-2.json</t>
-        </is>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>DATA-09</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>Secrets Manager secrets rotate automatically</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>CC6.1</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>us-west-2</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>No resources in scope</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="inlineStr">
-        <is>
-          <t>Configure a rotation Lambda and schedule for the secret.</t>
-        </is>
-      </c>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>evidence/DATA-09__us-west-2.json</t>
-        </is>
-      </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>LOG-08</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Log groups retain logs for at least 365 days</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>CC7.2</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>us-west-2</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>No resources in scope</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>Set retention to 365+ days (or 'never expire') on each log group.</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>evidence/LOG-08__us-west-2.json</t>
-        </is>
-      </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26T14:42:51Z</t>
+          <t>evidence/NET-02__us-east-1.json, evidence/NET-02__us-west-2.json</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J48"/>
+  <autoFilter ref="A1:H32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence file</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Evaluated (UTC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>DATA-07</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>RDS databases are not publicly accessible</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>us-east-1</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>1 of 2 failing</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>evidence/DATA-07__us-east-1.json</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>IAM-01</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Root account has MFA enabled</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 failing</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>evidence/IAM-01.json</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>NET-01</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>No security group exposes SSH or RDP to the internet</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>us-east-1</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>1 of 3 failing</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>evidence/NET-01__us-east-1.json</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>AVL-01</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>RDS automated backups are kept at least 7 days</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>us-east-1</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>1 of 2 failing</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>evidence/AVL-01__us-east-1.json</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>DATA-06</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>RDS databases are encrypted at rest</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>us-east-1</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>1 of 2 failing</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>evidence/DATA-06__us-east-1.json</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>IAM-04</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Every console user has MFA</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>1 of 2 failing</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>evidence/IAM-04.json</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>IAM-08</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>No customer-managed policy grants full admin (*:*)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>1 of 2 failing</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>evidence/IAM-08.json</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>LOG-04</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>AWS Config is recording</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>us-west-2</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 failing</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>evidence/LOG-04__us-west-2.json</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>LOG-05</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>GuardDuty is enabled</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>us-west-2</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 failing</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>evidence/LOG-05__us-west-2.json</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>AVL-02</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>RDS databases are Multi-AZ</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>us-east-1</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>1 of 2 failing</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>evidence/AVL-02__us-east-1.json</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>AVL-03</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>An AWS Backup plan exists</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>us-west-2</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 failing</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>evidence/AVL-03__us-west-2.json</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:10Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>DATA-03</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>S3 buckets reject non-TLS requests</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>1 of 4 failing</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>evidence/DATA-03.json</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:10Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>DATA-05</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>EBS encryption by default is on</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>us-west-2</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 failing</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>evidence/DATA-05__us-west-2.json</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:10Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>DATA-08</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Customer-managed KMS keys rotate automatically</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>us-east-1</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>1 of 2 failing</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>evidence/DATA-08__us-east-1.json</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>IAM-03</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Password policy meets minimum strength</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 failing</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>evidence/IAM-03.json</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>LOG-06</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Security Hub is enabled</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>us-west-2</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 failing</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>evidence/LOG-06__us-west-2.json</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>LOG-07</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Every VPC has flow logs</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>us-west-2</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 failing</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>evidence/LOG-07__us-west-2.json</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>DATA-04</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>S3 buckets have versioning enabled</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>1 of 4 failing</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>evidence/DATA-04.json</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:10Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>DATA-09</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Secrets Manager secrets rotate automatically</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>us-east-1</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 failing</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>evidence/DATA-09__us-east-1.json</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>IAM-07</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>IAM users get permissions through groups or roles only</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>1 of 3 failing</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>evidence/IAM-07.json</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>LOG-03</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>CloudTrail logs are encrypted with KMS</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 failing</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>evidence/LOG-03.json</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>LOG-08</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Log groups retain logs for at least 365 days</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>us-east-1</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>1 of 2 failing</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>evidence/LOG-08__us-east-1.json</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>IAM-09</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>IAM Access Analyzer is enabled</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>us-east-1</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Check could not be evaluated (The AWS simulator used for this sample does not support this API.)</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>evidence/IAM-09__us-east-1.json</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>IAM-09</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>IAM Access Analyzer is enabled</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>us-west-2</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Check could not be evaluated (The AWS simulator used for this sample does not support this API.)</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>evidence/IAM-09__us-west-2.json</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>DATA-02</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>No S3 bucket allows public access</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>4 of 4 passing</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>evidence/DATA-02.json</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:10Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>IAM-02</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Root account has no access keys</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>evidence/IAM-02.json</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>LOG-01</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>A multi-region CloudTrail trail is logging</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>evidence/LOG-01.json</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>NET-01</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>No security group exposes SSH or RDP to the internet</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>us-west-2</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>evidence/NET-01__us-west-2.json</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>DATA-01</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>S3 Block Public Access is on at the account level</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>evidence/DATA-01.json</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:10Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>LOG-04</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>AWS Config is recording</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>us-east-1</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>evidence/LOG-04__us-east-1.json</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>LOG-05</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>GuardDuty is enabled</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>us-east-1</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>evidence/LOG-05__us-east-1.json</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>AVL-03</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>An AWS Backup plan exists</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>us-east-1</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>evidence/AVL-03__us-east-1.json</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:10Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>DATA-05</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>EBS encryption by default is on</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>us-east-1</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>evidence/DATA-05__us-east-1.json</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:10Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>IAM-05</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Access keys are rotated within 90 days</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>evidence/IAM-05.json</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:13Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>IAM-06</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Unused credentials are disabled</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>3 of 3 passing</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>evidence/IAM-06.json</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>LOG-02</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>CloudTrail log file validation is enabled</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>evidence/LOG-02.json</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>LOG-06</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Security Hub is enabled</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>us-east-1</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>evidence/LOG-06__us-east-1.json</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>LOG-07</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Every VPC has flow logs</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>us-east-1</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>evidence/LOG-07__us-east-1.json</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>NET-02</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Default security groups allow no traffic</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>us-east-1</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>evidence/NET-02__us-east-1.json</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>NET-02</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Default security groups allow no traffic</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>us-west-2</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1 passing</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>evidence/NET-02__us-west-2.json</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>DATA-07</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>RDS databases are not publicly accessible</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>us-west-2</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>No resources in scope</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>evidence/DATA-07__us-west-2.json</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>AVL-01</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>RDS automated backups are kept at least 7 days</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>us-west-2</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>No resources in scope</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>evidence/AVL-01__us-west-2.json</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>DATA-06</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>RDS databases are encrypted at rest</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>us-west-2</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>No resources in scope</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>evidence/DATA-06__us-west-2.json</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>AVL-02</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>RDS databases are Multi-AZ</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>us-west-2</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>No resources in scope</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>evidence/AVL-02__us-west-2.json</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>DATA-08</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Customer-managed KMS keys rotate automatically</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>us-west-2</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>No resources in scope</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>evidence/DATA-08__us-west-2.json</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>DATA-09</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Secrets Manager secrets rotate automatically</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>us-west-2</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>No resources in scope</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>evidence/DATA-09__us-west-2.json</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>LOG-08</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Log groups retain logs for at least 365 days</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>us-west-2</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>No resources in scope</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>evidence/LOG-08__us-west-2.json</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26T15:22:11Z</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G48"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3252,7 +3912,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>sg-3e9e2eb22fcf9f64b (bastion)</t>
+          <t>sg-66222b5123eb54f73 (bastion)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -3604,7 +4264,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>arn:aws:kms:us-east-1:123456789012:key/34298638-74ad-4425-8a87-bf9d4429585e</t>
+          <t>arn:aws:kms:us-east-1:123456789012:key/796fe191-66ff-4c30-b1bc-7e6d8fc811b2</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -3700,7 +4360,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>vpc-6b2c3f62ea0a4b193</t>
+          <t>vpc-dd05bc29cc33c0616</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -3764,7 +4424,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>arn:aws:secretsmanager:us-east-1:123456789012:secret:prod/patients-db-ShzdBB</t>
+          <t>arn:aws:secretsmanager:us-east-1:123456789012:secret:prod/patients-db-LYNLUp</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -3885,7 +4545,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4733,7 +5393,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5052,16 +5712,16 @@
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>8</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -5210,7 +5870,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F15" s="2" t="n">
         <v>2</v>
@@ -5219,7 +5879,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -5274,7 +5934,7 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17" s="2" t="n">
         <v>1</v>
@@ -5308,13 +5968,13 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F18" s="2" t="n">
         <v>2</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>0</v>
@@ -5338,7 +5998,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F19" s="2" t="n">
         <v>4</v>
@@ -5347,7 +6007,7 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -5436,7 +6096,7 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
         <v>1</v>
@@ -5526,7 +6186,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25" s="2" t="n">
         <v>4</v>
@@ -5535,7 +6195,7 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -5586,7 +6246,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F27" s="2" t="n">
         <v>3</v>
@@ -5595,7 +6255,7 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">

</xml_diff>

<commit_message>
Tighten two checks after the first real-account scan
Reviewed a 17-region scan of a real account: no false positives, but two
results were less precise than they should be.

- DATA-02 measured Block Public Access coverage but was titled as if it
  proved buckets were public. Renamed to say what it checks.
- NET-01 now says whether each open security group is attached to
  anything, so unused groups read as "safe to delete" (adds the read-only
  ec2:DescribeNetworkInterfaces permission; policy and templates updated).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017pwRQCbGzSVKnLyfg31ziv
</commit_message>
<xml_diff>
--- a/web/sample/workbook.xlsx
+++ b/web/sample/workbook.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:10Z</t>
+          <t>2026-10-26T15:36:26Z</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:13Z</t>
+          <t>2026-10-26T15:36:29Z</t>
         </is>
       </c>
     </row>
@@ -795,7 +795,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Remove the open rule; use SSM Session Manager or a VPN / bastion with a narrow source range.</t>
+          <t>Remove the open rule; use SSM Session Manager or a VPN / bastion with a narrow source range. Groups not attached to anything can simply be deleted.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>No S3 bucket allows public access</t>
+          <t>Every S3 bucket is protected by Block Public Access</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2148,7 +2148,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2185,7 +2185,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:28Z</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2222,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2259,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2333,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2370,7 +2370,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2407,7 +2407,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2444,7 +2444,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:10Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2481,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:10Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2518,7 +2518,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:10Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2555,7 +2555,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2592,7 +2592,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2629,7 +2629,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:28Z</t>
         </is>
       </c>
     </row>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2703,7 +2703,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:10Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2740,7 +2740,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2814,7 +2814,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2888,7 +2888,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2925,7 +2925,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>No S3 bucket allows public access</t>
+          <t>Every S3 bucket is protected by Block Public Access</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2962,7 +2962,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:10Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -3036,7 +3036,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -3073,7 +3073,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -3110,7 +3110,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:10Z</t>
+          <t>2026-10-26T15:36:26Z</t>
         </is>
       </c>
     </row>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -3184,7 +3184,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -3221,7 +3221,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:10Z</t>
+          <t>2026-10-26T15:36:26Z</t>
         </is>
       </c>
     </row>
@@ -3258,7 +3258,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:10Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:13Z</t>
+          <t>2026-10-26T15:36:29Z</t>
         </is>
       </c>
     </row>
@@ -3332,7 +3332,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -3369,7 +3369,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -3406,7 +3406,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3517,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3554,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -3591,7 +3591,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -3628,7 +3628,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:28Z</t>
         </is>
       </c>
     </row>
@@ -3702,7 +3702,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -3739,7 +3739,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -3776,7 +3776,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T15:22:11Z</t>
+          <t>2026-10-26T15:36:27Z</t>
         </is>
       </c>
     </row>
@@ -3912,7 +3912,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>sg-66222b5123eb54f73 (bastion)</t>
+          <t>sg-6849222529ab1c680 (bastion)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -3922,12 +3922,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Open to internet: SSH (22)</t>
+          <t>Open to internet: SSH (22) (not attached to anything, safe to delete)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Remove the open rule; use SSM Session Manager or a VPN / bastion with a narrow source range.</t>
+          <t>Remove the open rule; use SSM Session Manager or a VPN / bastion with a narrow source range. Groups not attached to anything can simply be deleted.</t>
         </is>
       </c>
     </row>
@@ -4264,7 +4264,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>arn:aws:kms:us-east-1:123456789012:key/796fe191-66ff-4c30-b1bc-7e6d8fc811b2</t>
+          <t>arn:aws:kms:us-east-1:123456789012:key/c14e29de-6356-4a5e-aafc-4fbd388bbb1f</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -4360,7 +4360,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>vpc-dd05bc29cc33c0616</t>
+          <t>vpc-f1b8fce8c8b7057a1</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -4424,7 +4424,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>arn:aws:secretsmanager:us-east-1:123456789012:secret:prod/patients-db-LYNLUp</t>
+          <t>arn:aws:secretsmanager:us-east-1:123456789012:secret:prod/patients-db-tkjfqW</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">

</xml_diff>